<commit_message>
ampex crt and misc
</commit_message>
<xml_diff>
--- a/ampex-d175-terminal/digital-to-crt-pinout.xlsx
+++ b/ampex-d175-terminal/digital-to-crt-pinout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matt\Dropbox\Projects\serial-terminals\ampex-d175-terminal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575B192A-74AA-4E6F-A13A-6A118C98BD62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9256EA-86B8-469F-9BE2-651122028A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6960" yWindow="1725" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="945" yWindow="2295" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="73">
   <si>
     <t>Pin</t>
   </si>
@@ -106,6 +106,144 @@
   </si>
   <si>
     <t>Unreg V+ 10.9V</t>
+  </si>
+  <si>
+    <t>12v rail caps</t>
+  </si>
+  <si>
+    <t>C110</t>
+  </si>
+  <si>
+    <t>C311</t>
+  </si>
+  <si>
+    <t>C204</t>
+  </si>
+  <si>
+    <t>Missing</t>
+  </si>
+  <si>
+    <t>Unreg Pre-12v</t>
+  </si>
+  <si>
+    <t>C108</t>
+  </si>
+  <si>
+    <t>3300uf  35v</t>
+  </si>
+  <si>
+    <t>Axial</t>
+  </si>
+  <si>
+    <t>Unreg pre 5v</t>
+  </si>
+  <si>
+    <t>C107</t>
+  </si>
+  <si>
+    <t>10000uf 25v</t>
+  </si>
+  <si>
+    <t>Pre-fix:</t>
+  </si>
+  <si>
+    <t>5v rail</t>
+  </si>
+  <si>
+    <t>pre-reg 5v @ C107</t>
+  </si>
+  <si>
+    <t>~ 120hz, 0.77 ripple, 10.9v</t>
+  </si>
+  <si>
+    <t>66 mV ripple, 5.02v</t>
+  </si>
+  <si>
+    <t>12v rail</t>
+  </si>
+  <si>
+    <t>pre-reg 12v @ C108</t>
+  </si>
+  <si>
+    <t>~ 120hz, 1.6v ripple, 21.4v</t>
+  </si>
+  <si>
+    <t>191 mV ripple, 11.85v</t>
+  </si>
+  <si>
+    <t>Full screen</t>
+  </si>
+  <si>
+    <t>1.9 V</t>
+  </si>
+  <si>
+    <t>235 mV</t>
+  </si>
+  <si>
+    <t>~ 0.5v when looked at 20 us/div</t>
+  </si>
+  <si>
+    <t>C501</t>
+  </si>
+  <si>
+    <t>C502</t>
+  </si>
+  <si>
+    <t>100uF 35v</t>
+  </si>
+  <si>
+    <t>C109</t>
+  </si>
+  <si>
+    <t>1uF 50v</t>
+  </si>
+  <si>
+    <t>220 uF 16v</t>
+  </si>
+  <si>
+    <t>C303</t>
+  </si>
+  <si>
+    <t>0.47uF 50v</t>
+  </si>
+  <si>
+    <t>C306</t>
+  </si>
+  <si>
+    <t>C301</t>
+  </si>
+  <si>
+    <t>C304</t>
+  </si>
+  <si>
+    <t>10 uF 16v</t>
+  </si>
+  <si>
+    <t>47 uF 25v</t>
+  </si>
+  <si>
+    <t>C305</t>
+  </si>
+  <si>
+    <t>C307</t>
+  </si>
+  <si>
+    <t>2200 uF 16v</t>
+  </si>
+  <si>
+    <t>C205</t>
+  </si>
+  <si>
+    <t>25uF 25v non-polar ?</t>
+  </si>
+  <si>
+    <t>C503</t>
+  </si>
+  <si>
+    <t>100Uf 160v Axial</t>
+  </si>
+  <si>
+    <t>100uF 10v</t>
   </si>
 </sst>
 </file>
@@ -423,9 +561,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
     <col min="3" max="3" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -571,6 +710,204 @@
         <v>13</v>
       </c>
     </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D34" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>39</v>
+      </c>
+      <c r="E36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B37" t="s">
+        <v>41</v>
+      </c>
+      <c r="C37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>40</v>
+      </c>
+      <c r="C38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" t="s">
+        <v>46</v>
+      </c>
+      <c r="E39" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" t="s">
+        <v>47</v>
+      </c>
+      <c r="E40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F40" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>